<commit_message>
Update course analysis documents and Excel files for IKS and ISLL
- Modified course reference files for IKS and ISLL, updating the number of rows in Excel downloads.
- Added new problematic course plans and updated existing entries in Markdown files for IKS analysis.
- Corrected spelling errors and language consistency issues in course plans.
- Updated binary Excel files for various analyses, including grading reports and learning outcomes.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsrapportering.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsrapportering.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Betygsrapportering" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsrapportering'!$A$1:$E$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsrapportering'!$A$1:$E$168</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,12 +472,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ABY22V</t>
+          <t>FDA222R</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,24 +487,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY22V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222R</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ABY22W</t>
+          <t>FDA222S</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -514,24 +514,24 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY22W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222S</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ABY27W</t>
+          <t>FDA222T</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -541,24 +541,24 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY27W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222T</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BY1047</t>
+          <t>FDA222U</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -568,19 +568,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Två projektuppgifter om 3,5 respektive 4 hp. Två seminarier om 4 respektive 3,5 hp För godk…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1047</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222U</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BY1053</t>
+          <t>ABY22V</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -595,19 +595,19 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift U-G.…</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1053</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY22V</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BY1054</t>
+          <t>ABY22W</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -622,19 +622,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen bestäms av den skriftliga tentamen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1054</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY22W</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>BY1056</t>
+          <t>ABY27W</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -649,19 +649,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer U-G. Betygssättningen av kursen sker efter bedömning av den skriftliga …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1056</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ABY27W</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>BY1058</t>
+          <t>BY1047</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -676,19 +676,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Två projektuppgifter om 3,5 respektive 4 hp. Två seminarier om 4 respektive 3,5 hp För godk…</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1058</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1047</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>BY1059</t>
+          <t>BY1053</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -703,19 +703,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1053</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>BY1061</t>
+          <t>BY1054</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -730,19 +730,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projekt med skriftlig redovisning och seminarium (G/U) Betyget på skriftlig tentamen…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen bestäms av den skriftliga tentamen.…</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1061</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1054</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>BY1065</t>
+          <t>BY1056</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -757,19 +757,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig redovisning av projektuppgift och skriftlig inlämningsuppgift, U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer U-G. Betygssättningen av kursen sker efter bedömning av den skriftliga …</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1065</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1056</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>BY2016</t>
+          <t>BY1058</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -784,19 +784,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Arbetet måste senast vara klart inom 18 månader från kursstart annars ges examensarb…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2016</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1058</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BY2022</t>
+          <t>BY1059</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift (poster och reflektionsprotokoll) U, 3, 4, 5 Laborationer och semi…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>BY2025</t>
+          <t>BY1061</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -838,19 +838,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projekt med skriftlig redovisning och seminarium (G/U) Betyget på skriftlig tentamen…</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1061</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>BY3001</t>
+          <t>BY1065</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -865,19 +865,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig redovisning av projektuppgift och skriftlig inlämningsuppgift, U-G.…</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1065</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>BY3004</t>
+          <t>BY2016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -892,19 +892,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Arbetet måste senast vara klart inom 18 månader från kursstart annars ges examensarb…</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2016</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BY3005</t>
+          <t>BY2022</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -919,19 +919,19 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Reflektionsprotokoll ges betyget (U-G). Seminarier ges betyget (U-VG). Slutbetyg sät…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift (poster och reflektionsprotokoll) U, 3, 4, 5 Laborationer och semi…</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GBY2GB</t>
+          <t>BY2025</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -951,14 +951,14 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2GB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2025</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GBY2GC</t>
+          <t>BY3001</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -973,19 +973,19 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig tentamen, U-3-4-5. Seminarier, U-G. Skriftlig inlämningsuppgift, U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2GC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3001</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>GBY2GR</t>
+          <t>BY3004</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1000,19 +1000,19 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Litteraturseminarium och laborationer U-G. Slutbetyget sätts efter en samlad bedömni…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2GR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3004</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>GBY2J2</t>
+          <t>BY3005</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1027,19 +1027,19 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig deltentamen 1, U,3,4,5 Projektuppgift, U-VG Skriftlig deltentamen 2, U,3,4…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Reflektionsprotokoll ges betyget (U-G). Seminarier ges betyget (U-VG). Slutbetyg sät…</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2J2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>GBY2MA</t>
+          <t>GBY2GB</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1054,19 +1054,19 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektuppgifter godkänd/underkänd Betyget på skriftlig tentamen utgör betyg på kurs…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2MA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2GB</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>GBY2MB</t>
+          <t>GBY2GC</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1081,19 +1081,19 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektuppgifter U-G. Individuellt PM U-VG. Seminarier U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig tentamen, U-3-4-5. Seminarier, U-G. Skriftlig inlämningsuppgift, U-G.…</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2MB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2GC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>GBY2ME</t>
+          <t>GBY2GR</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Kursbetyget baseras på tentamen U, 3, 4 ,5 Inlämningsuppgift och laboration U,G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Litteraturseminarium och laborationer U-G. Slutbetyget sätts efter en samlad bedömni…</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2ME</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2GR</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GBY2NF</t>
+          <t>GBY2J2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1135,19 +1135,19 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig tentamen U-3-4-5 Projektuppgift U-G Betyget på skriftlig tentamen utgör be…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig deltentamen 1, U,3,4,5 Projektuppgift, U-VG Skriftlig deltentamen 2, U,3,4…</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2NF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2J2</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GBY2NG</t>
+          <t>GBY2MA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1162,19 +1162,19 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgifter, seminarier och laborationer U,G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektuppgifter godkänd/underkänd Betyget på skriftlig tentamen utgör betyg på kurs…</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2NG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2MA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GBY2RN</t>
+          <t>GBY2MB</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig tentamen (U-3-4-5) Projekt (U-G) Betyget på skriftlig tentamen styr slutbe…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektuppgifter U-G. Individuellt PM U-VG. Seminarier U-G.…</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2MB</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GBY2RX</t>
+          <t>GBY2ME</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1216,19 +1216,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Betyget på skriftlig tentamen styr slutbetyget på kursen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Kursbetyget baseras på tentamen U, 3, 4 ,5 Inlämningsuppgift och laboration U,G.…</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2ME</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>GBY2V5</t>
+          <t>GBY2NF</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1243,19 +1243,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Salstentamen U,3,4,5 Projekt U/G Laborationsredovisning U/G Seminarier U/G…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig tentamen U-3-4-5 Projektuppgift U-G Betyget på skriftlig tentamen utgör be…</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2NF</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GBY2V6</t>
+          <t>GBY2NG</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1270,19 +1270,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgifter, seminarier och laborationer U,G.…</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2NG</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GBY2V8</t>
+          <t>GBY2RN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1297,19 +1297,19 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig tentamen (U-3-4-5) Projekt (U-G) Betyget på skriftlig tentamen styr slutbe…</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RN</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GBY2VR</t>
+          <t>GBY2RX</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1324,19 +1324,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projekt samt muntlig redovisning, U-VG Inlämningsuppgift samt seminarium, U-VG Seminarium,…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Betyget på skriftlig tentamen styr slutbetyget på kursen.…</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2VR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2RX</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GBY2XF</t>
+          <t>GBY2V5</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1351,24 +1351,24 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektuppgift U-VG Laboaration U-G Slutbetyget på kursen sätts efter en sammanvägni…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Salstentamen U,3,4,5 Projekt U/G Laborationsredovisning U/G Seminarier U/G…</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2XF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V5</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GDT2JM</t>
+          <t>GBY2V6</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DTA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1383,19 +1383,19 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V6</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GDT2JN</t>
+          <t>GBY2V8</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DTA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1405,24 +1405,24 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2V8</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ET1029</t>
+          <t>GBY2VR</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ETA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1432,24 +1432,24 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För laborationer ges betyg godkänd/underkänd.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projekt samt muntlig redovisning, U-VG Inlämningsuppgift samt seminarium, U-VG Seminarium,…</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2VR</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>BFY224</t>
+          <t>GBY2XF</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>FYA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1459,24 +1459,24 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Skriftlig rapport och muntlig redovisning 5 fup.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektuppgift U-VG Laboaration U-G Slutbetyget på kursen sätts efter en sammanvägni…</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BFY224</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY2XF</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>FY1018</t>
+          <t>GDT2JM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>FYA</t>
+          <t>DTA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1486,24 +1486,24 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer U,G Slutbetyg på kursen sätts efter bedömning av den skriftliga tentame…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JM</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GIE26L</t>
+          <t>GDT2JN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>DTA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1513,24 +1513,24 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDT2JN</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GIE26M</t>
+          <t>FEB222K</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1540,24 +1540,24 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222K</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GIE26N</t>
+          <t>FEB222L</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1567,24 +1567,24 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På skriftlig tentamen ges betyget U-3-4-5 På individuella inlämningsuppgifter ges be…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. För betyget godkänd på kursen krävs Godkänt på alla momenten listade nedan. Aktivt deltagan…</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222L</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GIE26P</t>
+          <t>FEB222M</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1594,24 +1594,24 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222M</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GIE29N</t>
+          <t>FEB222P</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1621,24 +1621,24 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222P</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GIE2L7</t>
+          <t>FEB222Q</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1648,24 +1648,24 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Betyg rapporteras enligt följande: Forskningsplan 2 hp Manus 2,5 hp Individuell rapport, 0,…</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2L7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GIE2MF</t>
+          <t>ET1029</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>ETA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1675,24 +1675,24 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För laborationer ges betyg godkänd/underkänd.…</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GIE2QS</t>
+          <t>BFY224</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>FYA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1702,24 +1702,24 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projekt, U-3-4-5 Inlämningsuppgifter, U-3-4-5 Slutbetyget på kursen ges av en samman…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Skriftlig rapport och muntlig redovisning 5 fup.…</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2QS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BFY224</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GIE2RF</t>
+          <t>FY1018</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>FYA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1729,19 +1729,19 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer U,G Slutbetyg på kursen sätts efter bedömning av den skriftliga tentame…</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2RF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>IE1068</t>
+          <t>GIE26L</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1756,19 +1756,19 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26L</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>IE1069</t>
+          <t>GIE26M</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1783,19 +1783,19 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På Mom 2 och 3 ges betyget U-G. Den skriftliga tentamen styr slutbetyget på kursen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26M</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>IE1076</t>
+          <t>GIE26N</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1810,19 +1810,19 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På inlämningsuppgiften ges betyget U-G Den skriftliga tentamen styr slutbetyget på k…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På skriftlig tentamen ges betyget U-3-4-5 På individuella inlämningsuppgifter ges be…</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1076</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26N</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>IE2003</t>
+          <t>GIE26P</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1837,24 +1837,24 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget sätts individuellt.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE2003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>AIK232</t>
+          <t>GIE29N</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1864,24 +1864,24 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig redovisning av laborationer U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GIK23M</t>
+          <t>GIE2L7</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1891,24 +1891,24 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Resultatet på den skriftliga tentamen styr slutbetyget på kursen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2L7</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GIK289</t>
+          <t>GIE2MF</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1918,24 +1918,24 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GIK299</t>
+          <t>GIE2QS</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1945,24 +1945,24 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projekt, U-3-4-5 Inlämningsuppgifter, U-3-4-5 Slutbetyget på kursen ges av en samman…</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK299</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2QS</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GIK2AL</t>
+          <t>GIE2RF</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1972,24 +1972,24 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2AL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2RF</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>GIK2BD</t>
+          <t>IE1068</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1999,24 +1999,24 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2BD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1068</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>GIK2FB</t>
+          <t>IE1069</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2026,24 +2026,24 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laboration U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På Mom 2 och 3 ges betyget U-G. Den skriftliga tentamen styr slutbetyget på kursen.…</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2FB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>GIK2JX</t>
+          <t>IE1076</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2053,24 +2053,24 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarier U-G. Slutbetyget baseras på sammanvägning av de examinerande momenten.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På inlämningsuppgiften ges betyget U-G Den skriftliga tentamen styr slutbetyget på k…</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2JX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1076</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>GIK2KM</t>
+          <t>IE2003</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2080,19 +2080,19 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter och duggor.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget sätts individuellt.…</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2KM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE2003</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>GIK2LF</t>
+          <t>AIK232</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2107,19 +2107,19 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig redovisning av laborationer U-G.…</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2LF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>GIK2NV</t>
+          <t>GIK23M</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2134,19 +2134,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget fastställs genom inlämningsuppgiften.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Resultatet på den skriftliga tentamen styr slutbetyget på kursen.…</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GIK2NX</t>
+          <t>GIK289</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2161,19 +2161,19 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor (U - VG), Laborationsredovisningar (U - G) och inlämningsuppgifter (U - VG). Slutbe…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>GIK2PB</t>
+          <t>GIK299</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2188,19 +2188,19 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarieuppgifter U-VG Projektarbete och laboration U-G För att erhålla slutbetyget VG på…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK299</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>GIK2AL</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2215,19 +2215,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på hela kursen krävs VG på projektuppgiften samt minst tv…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2AL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>GIK2PF</t>
+          <t>GIK2BD</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2242,19 +2242,19 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig tentamen 1,5hp U-VG, seminarier 3hp U-G, laborationer 3hp U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2BD</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GIK2PG</t>
+          <t>GIK2FB</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laboration U-G.…</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2FB</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GIK2Q3</t>
+          <t>GIK2JX</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2296,19 +2296,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U, G, VG), redovisning av laborationer (U,G) respektive seminarier (U,G).…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarier U-G. Slutbetyget baseras på sammanvägning av de examinerande momenten.…</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2JX</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>GIK2QZ</t>
+          <t>GIK2KM</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2323,19 +2323,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter och duggor.…</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2QZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2KM</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GIK2UK</t>
+          <t>GIK2LF</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2355,14 +2355,14 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2UK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2LF</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GIK2V4</t>
+          <t>GIK2NV</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget fastställs genom inlämningsuppgiften.…</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NV</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GIK2XJ</t>
+          <t>GIK2NX</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor, U-VG Seminarier, U-G Projekt, U-VG Slutbetyget på kursen baseras på en helhetsbedö…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor (U - VG), Laborationsredovisningar (U - G) och inlämningsuppgifter (U - VG). Slutbe…</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NX</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GIK2XK</t>
+          <t>GIK2PB</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarieuppgifter U-VG Projektarbete och laboration U-G För att erhålla slutbetyget VG på…</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PB</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GIK2XZ</t>
+          <t>GIK2PD</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2458,19 +2458,19 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på hela kursen krävs VG på projektuppgiften samt minst tv…</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>IK1032</t>
+          <t>GIK2PF</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2485,19 +2485,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig tentamen 1,5hp U-VG, seminarier 3hp U-G, laborationer 3hp U-G.…</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PF</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>GIK2PG</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2512,19 +2512,19 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter, laborati…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PG</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>IK1066</t>
+          <t>GIK2Q3</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2539,24 +2539,24 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För seminarer används betygsskalan U-G samt för dugga och projektarbete betygsskalan U-VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U, G, VG), redovisning av laborationer (U,G) respektive seminarier (U,G).…</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>GMA28W</t>
+          <t>GIK2QZ</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2566,24 +2566,24 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA28W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2QZ</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GMA2EY</t>
+          <t>GIK2UK</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2598,19 +2598,19 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2UK</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>MA0011</t>
+          <t>GIK2V4</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2620,24 +2620,24 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen kräva att alla examinerande moment är godkän…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>MA0013</t>
+          <t>GIK2XJ</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2647,24 +2647,24 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen krävs att alla examinerande moment är godkän…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor, U-VG Seminarier, U-G Projekt, U-VG Slutbetyget på kursen baseras på en helhetsbedö…</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XJ</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>MA1040</t>
+          <t>GIK2XK</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2674,24 +2674,24 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg på kursen avgörs efter en sammanvägd bedömning av de enskilda tentamensres…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XK</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>MA1042</t>
+          <t>GIK2XZ</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2701,24 +2701,24 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XZ</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>IK1032</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2728,24 +2728,24 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla väl godkänt på kursen krävs väl godkänt som bedömning på 3 av 4 skriftliga…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2755,24 +2755,24 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,G Workshop och inlämningsuppgifter, U,G. Seminarier U, 3,4,5 Skriftl…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter, laborati…</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>GMT25Z</t>
+          <t>IK1066</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2782,24 +2782,24 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För seminarer används betygsskalan U-G samt för dugga och projektarbete betygsskalan U-VG.…</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>GMA28W</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2809,24 +2809,24 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA28W</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>MT1033</t>
+          <t>GMA2EY</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2841,19 +2841,19 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>MA0011</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2863,24 +2863,24 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen kräva att alla examinerande moment är godkän…</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0011</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>MA0013</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2890,24 +2890,24 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Industriprojekt och workshop, U,G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen krävs att alla examinerande moment är godkän…</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0013</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>MT1074</t>
+          <t>MA1040</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2917,24 +2917,24 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer samt laborationsrapporter U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg på kursen avgörs efter en sammanvägd bedömning av de enskilda tentamensres…</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1040</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>MA1042</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2949,19 +2949,19 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2971,24 +2971,24 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla väl godkänt på kursen krävs väl godkänt som bedömning på 3 av 4 skriftliga…</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>FMI2222</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2998,24 +2998,24 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntliga presentationer och skriftliga grupprapporter för projektet, U-G. Det samlade bety…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>FMI2223</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3025,24 +3025,24 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2223</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>AEG26X</t>
+          <t>FMI2224</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3052,24 +3052,24 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift 1: 2 hp, U-G Inlämningsuppgift 2: 3 hp, U, 3, 4, 5 Inlämningsuppgi…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>BEG222</t>
+          <t>FMI2229</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3084,19 +3084,19 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2229</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>EG1012</t>
+          <t>MIKR002</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3106,24 +3106,24 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts av examinator efter en sammanvägning av momenten.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Betygsrapportering: Moment 1: enskilt projekt 2 hp Moment 2: laborationsrapporter 1 hp Mome…</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MIKR002</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>EG2004</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3133,24 +3133,24 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Arbetet måste senast vara klart inom 18 månader från kursstart annars ges examensarb…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,G Workshop och inlämningsuppgifter, U,G. Seminarier U, 3,4,5 Skriftl…</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG2004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>GMT25Z</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3160,24 +3160,24 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationsrapporter (U, G) Betyget för hela kursen sätts efter en samlad bedömning …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>EG3009</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -3187,24 +3187,24 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig hemuppgift 1, U-G. Slutbetyget sätts efter en samlad bedömning av examinat…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>EG3012</t>
+          <t>MT1033</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -3214,24 +3214,24 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget för kursen är baserad på betyget för tentan…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -3241,24 +3241,24 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter bedömning av reflektionsprotokoll. Väl genomförda skriftliga r…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3268,24 +3268,24 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Reflektionsprotokoll, skriftlig rapport och projektuppgift (U-G). Den skiftliga tent…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Industriprojekt och workshop, U,G.…</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>EG3017</t>
+          <t>MT1074</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -3295,24 +3295,24 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer samt laborationsrapporter U-G.…</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>EG3018</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3322,19 +3322,19 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>EG3019</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3349,19 +3349,19 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laboration och Inlämningsuppgifter U,G…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3019</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>EG3020</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3376,19 +3376,19 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntliga presentationer och skriftliga grupprapporter för projektet, U-G. Det samlade bety…</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>EG3022</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3403,19 +3403,19 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>EG4001</t>
+          <t>AEG26X</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3430,19 +3430,19 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift 1: 2 hp, U-G Inlämningsuppgift 2: 3 hp, U, 3, 4, 5 Inlämningsuppgi…</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>BEG222</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3462,14 +3462,14 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>GEG2JP</t>
+          <t>EG1012</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3484,19 +3484,19 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift, rapport och muntlig presentation ger U eller G. Det samlade betyg…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts av examinator efter en sammanvägning av momenten.…</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>GEG2UE</t>
+          <t>EG2004</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3511,19 +3511,19 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Rapporter (U/G) Betygssättning av kursen sker genom den skriftliga salstentamen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Arbetet måste senast vara klart inom 18 månader från kursstart annars ges examensarb…</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG2004</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>GEG2UL</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3538,24 +3538,24 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntlig redovisning U-G. Projekt U-VG. Kursens slutbetyg baseras på en samlad bedömning av…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationsrapporter (U, G) Betyget för hela kursen sätts efter en samlad bedömning …</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>GSQ23J</t>
+          <t>EG3009</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3565,24 +3565,24 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig hemuppgift 1, U-G. Slutbetyget sätts efter en samlad bedömning av examinat…</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>EG3012</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3592,24 +3592,24 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,VG Slutbetyget på kursen sätts efter en samlad bedömning av examinat…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget för kursen är baserad på betyget för tentan…</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>GSQ25F</t>
+          <t>EG3014</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3619,24 +3619,24 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete och övningsuppgifter U,VG. Slutbetyget utgör en sammanvägning av betyg…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter bedömning av reflektionsprotokoll. Väl genomförda skriftliga r…</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>GSQ25J</t>
+          <t>EG3015</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3646,24 +3646,24 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Reflektionsprotokoll, skriftlig rapport och projektuppgift (U-G). Den skiftliga tent…</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>GSQ25K</t>
+          <t>EG3017</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3673,24 +3673,24 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För projektarbetet är betygsskalan U,G,VG. Slutbetyget på kursen sätts efter en saml…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>GSQ25N</t>
+          <t>EG3018</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3700,24 +3700,24 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>EG3019</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3727,24 +3727,24 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laboration och Inlämningsuppgifter U,G…</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3019</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>GSQ2H7</t>
+          <t>EG3020</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3754,24 +3754,24 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3020</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>GSQ2J4</t>
+          <t>EG3022</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3781,24 +3781,24 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som sammanvägd betygsskala används U, 3,4, 5 med följande fördelning på delmomenten:…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F.…</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L8</t>
+          <t>EG4001</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3808,24 +3808,24 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Tentamen och seminarier med skriftliga inlämningar, U, 3, 4, 5. Projektuppgiften, U,…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F.…</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3835,24 +3835,24 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>GSQ2LA</t>
+          <t>GEG2JP</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3862,24 +3862,24 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Tentamen och övningar, U-G. Seminarier och projektuppgift, U-VG. Slutbetyget på kursen sät…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift, rapport och muntlig presentation ger U eller G. Det samlade betyg…</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2LA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>GSQ2MC</t>
+          <t>GEG2UE</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3889,24 +3889,24 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Rapporter (U/G) Betygssättning av kursen sker genom den skriftliga salstentamen.…</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UE</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>GSQ2PH</t>
+          <t>GEG2UL</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3916,19 +3916,19 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som betygsskala för kursen och för tentamen används U, 3, 4, 5. För litteratursemina…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntlig redovisning U-G. Projekt U-VG. Kursens slutbetyg baseras på en samlad bedömning av…</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>GSQ2R5</t>
+          <t>GSQ23J</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3943,19 +3943,19 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U-VG) Övningar (U-G) Seminarier (U-G)…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2R5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>GSQ2VY</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3970,19 +3970,19 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektet styr slutbetyget på kursen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,VG Slutbetyget på kursen sätts efter en samlad bedömning av examinat…</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>GSQ2WM</t>
+          <t>GSQ25F</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3997,19 +3997,19 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på Modul 1 och Modul 2. Modul 1: Kartografi och …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete och övningsuppgifter U,VG. Slutbetyget utgör en sammanvägning av betyg…</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>GSQ2Y2</t>
+          <t>GSQ25J</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -4024,19 +4024,19 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på både Modul 1 och Modul 2. Modul 1: Kvalitativ…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2Y2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>SQ1003</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -4051,24 +4051,24 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För projektarbetet är betygsskalan U,G,VG. Slutbetyget på kursen sätts efter en saml…</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>GST2CL</t>
+          <t>GSQ25N</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -4078,24 +4078,24 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25N</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>ST1013</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -4110,19 +4110,19 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>AMI22T</t>
+          <t>GSQ2H7</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -4132,24 +4132,24 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>AMI22Z</t>
+          <t>GSQ2J4</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -4159,24 +4159,24 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som sammanvägd betygsskala används U, 3,4, 5 med följande fördelning på delmomenten:…</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>AMI23A</t>
+          <t>GSQ2L8</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -4186,24 +4186,24 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Tentamen och seminarier med skriftliga inlämningar, U, 3, 4, 5. Projektuppgiften, U,…</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>AMI23C</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -4213,24 +4213,24 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>AMI23G</t>
+          <t>GSQ2LA</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -4240,24 +4240,24 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete U - VG Laborationer, seminarier och skriftlig reflektioner U-G. Slutbetyget …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Tentamen och övningar, U-G. Seminarier och projektuppgift, U-VG. Slutbetyget på kursen sät…</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2LA</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>AMI23J</t>
+          <t>GSQ2MC</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -4267,24 +4267,24 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>AMI23K</t>
+          <t>GSQ2PH</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -4294,24 +4294,24 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget på kursen sätts efter en samlad bedömning av examina…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som betygsskala för kursen och för tentamen används U, 3, 4, 5. För litteratursemina…</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>AMI23L</t>
+          <t>GSQ2R5</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -4321,24 +4321,24 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U-VG) Övningar (U-G) Seminarier (U-G)…</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2R5</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>AMI27V</t>
+          <t>GSQ2VY</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -4348,24 +4348,24 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektet styr slutbetyget på kursen.…</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI27V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>GMI23G</t>
+          <t>GSQ2WM</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -4375,24 +4375,24 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på Modul 1 och Modul 2. Modul 1: Kartografi och …</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>GMI24H</t>
+          <t>GSQ2Y2</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -4402,24 +4402,24 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Labborationsuppgifter U-G Salstentamen U-VG Kursens slutbetyg bestäms av betyget för salst…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på både Modul 1 och Modul 2. Modul 1: Kvalitativ…</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2Y2</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>GMI26H</t>
+          <t>SQ1003</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -4429,24 +4429,24 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betygets nivå fastställs genom tentamen, vilket också blir slutbetyget under förutsättning…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>GMI2C8</t>
+          <t>GST2CL</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4456,24 +4456,24 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>GMI2J3</t>
+          <t>ST1013</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -4483,19 +4483,19 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Inlämningsuppgifter och gruppresentation, U-G. Skriftlig tentamen, U-VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>GMI2MD</t>
+          <t>AMI22T</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4510,19 +4510,19 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Individuell muntlig och skriftlig redovisning av inlämningsuppgifter och gruppresentation …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GMI2NW</t>
+          <t>AMI22Z</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4542,14 +4542,14 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2NW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22Z</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>MI4001</t>
+          <t>AMI23A</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4564,44 +4564,422 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget är individuellt och sätts på grundval av det material som föreligger vid slutsemin…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
+          <t>AMI23C</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>AMI23G</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete U - VG Laborationer, seminarier och skriftlig reflektioner U-G. Slutbetyget …</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>AMI23J</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23J</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>AMI23K</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget på kursen sätts efter en samlad bedömning av examina…</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>AMI23L</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>AMI27V</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI27V</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>GMI23G</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>GMI24H</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Labborationsuppgifter U-G Salstentamen U-VG Kursens slutbetyg bestäms av betyget för salst…</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>GMI26H</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betygets nivå fastställs genom tentamen, vilket också blir slutbetyget under förutsättning…</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>GMI2C8</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>GMI2J3</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Inlämningsuppgifter och gruppresentation, U-G. Skriftlig tentamen, U-VG.…</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>GMI2MD</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Individuell muntlig och skriftlig redovisning av inlämningsuppgifter och gruppresentation …</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>GMI2NW</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2NW</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>MI4001</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget är individuellt och sätts på grundval av det material som föreligger vid slutsemin…</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
           <t>MI4002</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B168" t="inlineStr">
         <is>
           <t>XYZ</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Saknar punktlista</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
         <is>
           <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget är individuellt och sätts på grundval av det material som föreligger vid slutsemin…</t>
         </is>
       </c>
-      <c r="E154" s="2" t="inlineStr">
+      <c r="E168" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4002</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E154"/>
+  <autoFilter ref="A1:E168"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -4909,6 +5287,34 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E153" r:id="rId304"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A154" r:id="rId305"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E154" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A155" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E155" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A156" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E156" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A157" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E157" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A158" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E158" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A159" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E159" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A160" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E160" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A161" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E161" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A162" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E162" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A163" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E163" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A164" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E164" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A165" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E165" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A166" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E166" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A167" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E167" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A168" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E168" r:id="rId334"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add course plans for GTY3KJ and GTY3KK: German Grammar and Writing with AI
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Betygsrapportering.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Betygsrapportering.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Betygsrapportering" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsrapportering'!$A$1:$G$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Betygsrapportering'!$A$1:$G$169</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G168"/>
+  <dimension ref="A1:G169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1771,17 +1771,17 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>FEB222K</t>
+          <t>GDV3KY</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ENERGIBM</t>
+          <t>DVE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2022-09-13</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -1797,14 +1797,14 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDV3KY</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>FEB222L</t>
+          <t>FEB222K</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1825,19 +1825,19 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. För betyget godkänd på kursen krävs Godkänt på alla momenten listade nedan. Aktivt deltagan…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222K</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>FEB222M</t>
+          <t>FEB222L</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1858,19 +1858,19 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. För betyget godkänd på kursen krävs Godkänt på alla momenten listade nedan. Aktivt deltagan…</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222L</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>FEB222P</t>
+          <t>FEB222M</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2022-09-13</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1896,14 +1896,14 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222M</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>FEB222Q</t>
+          <t>FEB222P</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1924,29 +1924,29 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Betyg rapporteras enligt följande: Forskningsplan 2 hp Manus 2,5 hp Individuell rapport, 0,…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222P</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>ET1029</t>
+          <t>FEB222Q</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ETA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2018-02-13</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -1957,29 +1957,29 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För laborationer ges betyg godkänd/underkänd.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Betyg rapporteras enligt följande: Forskningsplan 2 hp Manus 2,5 hp Individuell rapport, 0,…</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BFY224</t>
+          <t>ET1029</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>FYA</t>
+          <t>ETA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2021-09-07</t>
+          <t>2018-02-13</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1990,19 +1990,19 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Skriftlig rapport och muntlig redovisning 5 fup.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För laborationer ges betyg godkänd/underkänd.…</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BFY224</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>FY1018</t>
+          <t>BFY224</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2017-06-15</t>
+          <t>2021-09-07</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -2023,29 +2023,29 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer U,G Slutbetyg på kursen sätts efter bedömning av den skriftliga tentame…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Skriftlig rapport och muntlig redovisning 5 fup.…</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BFY224</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GIE26L</t>
+          <t>FY1018</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>FYA</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2017-06-15</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -2056,19 +2056,19 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer U,G Slutbetyg på kursen sätts efter bedömning av den skriftliga tentame…</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GIE26M</t>
+          <t>GIE26L</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2089,19 +2089,19 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26L</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GIE26N</t>
+          <t>GIE26M</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2122,19 +2122,19 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På skriftlig tentamen ges betyget U-3-4-5 På individuella inlämningsuppgifter ges be…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26M</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GIE26P</t>
+          <t>GIE26N</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2155,19 +2155,19 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På skriftlig tentamen ges betyget U-3-4-5 På individuella inlämningsuppgifter ges be…</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26N</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GIE29N</t>
+          <t>GIE26P</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2019-06-13</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -2188,19 +2188,19 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GIE2L7</t>
+          <t>GIE29N</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2020-12-17</t>
+          <t>2019-06-13</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -2221,19 +2221,19 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På de individuella inlämningsuppgift…</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2L7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GIE2MF</t>
+          <t>GIE2L7</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2021-02-18</t>
+          <t>2020-12-17</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -2254,19 +2254,19 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5.…</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2L7</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GIE2QS</t>
+          <t>GIE2MF</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2276,7 +2276,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2021-06-17</t>
+          <t>2021-02-18</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -2287,19 +2287,19 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projekt, U-3-4-5 Inlämningsuppgifter, U-3-4-5 Slutbetyget på kursen ges av en samman…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På den skriftliga tentamen ges betyget U-3-4-5. På inlämningsuppgifterna ges betyget…</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2QS</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GIE2RF</t>
+          <t>GIE2QS</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2021-09-08</t>
+          <t>2021-06-17</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -2320,19 +2320,19 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projekt, U-3-4-5 Inlämningsuppgifter, U-3-4-5 Slutbetyget på kursen ges av en samman…</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2RF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2QS</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>IE1068</t>
+          <t>GIE2RF</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2015-02-05</t>
+          <t>2021-09-08</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -2353,19 +2353,19 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2RF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>IE1069</t>
+          <t>IE1068</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2386,19 +2386,19 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På Mom 2 och 3 ges betyget U-G. Den skriftliga tentamen styr slutbetyget på kursen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1068</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>IE1076</t>
+          <t>IE1069</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2018-03-08</t>
+          <t>2015-02-05</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -2419,19 +2419,19 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På inlämningsuppgiften ges betyget U-G Den skriftliga tentamen styr slutbetyget på k…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På Mom 2 och 3 ges betyget U-G. Den skriftliga tentamen styr slutbetyget på kursen.…</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1076</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>IE2003</t>
+          <t>IE1076</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2009-12-08</t>
+          <t>2018-03-08</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -2452,29 +2452,29 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget sätts individuellt.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. På inlämningsuppgiften ges betyget U-G Den skriftliga tentamen styr slutbetyget på k…</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE2003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1076</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AIK232</t>
+          <t>IE2003</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2019-04-29</t>
+          <t>2009-12-08</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -2485,19 +2485,19 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig redovisning av laborationer U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget sätts individuellt.…</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE2003</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>GIK23M</t>
+          <t>AIK232</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2018-08-23</t>
+          <t>2019-04-29</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -2518,19 +2518,19 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Resultatet på den skriftliga tentamen styr slutbetyget på kursen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig redovisning av laborationer U-G.…</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GIK289</t>
+          <t>GIK23M</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2018-08-23</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -2551,19 +2551,19 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Resultatet på den skriftliga tentamen styr slutbetyget på kursen.…</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>GIK299</t>
+          <t>GIK289</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2019-04-18</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -2589,14 +2589,14 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK299</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>GIK2AL</t>
+          <t>GIK299</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2019-08-29</t>
+          <t>2019-04-18</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -2622,14 +2622,14 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2AL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK299</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>GIK2BD</t>
+          <t>GIK2AL</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2639,7 +2639,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2019-09-11</t>
+          <t>2019-08-29</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -2655,14 +2655,14 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2BD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2AL</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GIK2FB</t>
+          <t>GIK2BD</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2672,7 +2672,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2020-03-05</t>
+          <t>2019-09-11</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -2683,19 +2683,19 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laboration U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2FB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2BD</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GIK2JX</t>
+          <t>GIK2FB</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2705,7 +2705,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2020-09-24</t>
+          <t>2020-03-05</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -2716,19 +2716,19 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarier U-G. Slutbetyget baseras på sammanvägning av de examinerande momenten.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laboration U-G.…</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2JX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2FB</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>GIK2KM</t>
+          <t>GIK2JX</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2749,19 +2749,19 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter och duggor.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarier U-G. Slutbetyget baseras på sammanvägning av de examinerande momenten.…</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2KM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2JX</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GIK2LF</t>
+          <t>GIK2KM</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2021-01-28</t>
+          <t>2020-09-24</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -2782,19 +2782,19 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter och duggor.…</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2LF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2KM</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GIK2NV</t>
+          <t>GIK2LF</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2021-03-11</t>
+          <t>2021-01-28</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -2815,19 +2815,19 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget fastställs genom inlämningsuppgiften.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2LF</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GIK2NX</t>
+          <t>GIK2NV</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2848,19 +2848,19 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor (U - VG), Laborationsredovisningar (U - G) och inlämningsuppgifter (U - VG). Slutbe…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget fastställs genom inlämningsuppgiften.…</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NV</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GIK2PB</t>
+          <t>GIK2NX</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
+          <t>2021-03-11</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -2881,19 +2881,19 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarieuppgifter U-VG Projektarbete och laboration U-G För att erhålla slutbetyget VG på…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor (U - VG), Laborationsredovisningar (U - G) och inlämningsuppgifter (U - VG). Slutbe…</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PB</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2NX</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>GIK2PB</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2914,19 +2914,19 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på hela kursen krävs VG på projektuppgiften samt minst tv…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Seminarieuppgifter U-VG Projektarbete och laboration U-G För att erhålla slutbetyget VG på…</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PB</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GIK2PF</t>
+          <t>GIK2PD</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2947,19 +2947,19 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig tentamen 1,5hp U-VG, seminarier 3hp U-G, laborationer 3hp U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på hela kursen krävs VG på projektuppgiften samt minst tv…</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>GIK2PG</t>
+          <t>GIK2PF</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2980,19 +2980,19 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Skriftlig tentamen 1,5hp U-VG, seminarier 3hp U-G, laborationer 3hp U-G.…</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PF</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>GIK2Q3</t>
+          <t>GIK2PG</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2021-05-20</t>
+          <t>2021-04-15</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -3013,19 +3013,19 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U, G, VG), redovisning av laborationer (U,G) respektive seminarier (U,G).…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PG</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>GIK2QZ</t>
+          <t>GIK2Q3</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2021-08-24</t>
+          <t>2021-05-20</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -3046,19 +3046,19 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U, G, VG), redovisning av laborationer (U,G) respektive seminarier (U,G).…</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2QZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2Q3</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GIK2UK</t>
+          <t>GIK2QZ</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2021-08-24</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
@@ -3084,14 +3084,14 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2UK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2QZ</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GIK2V4</t>
+          <t>GIK2UK</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3117,14 +3117,14 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2UK</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GIK2XJ</t>
+          <t>GIK2V4</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2022-09-06</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -3145,19 +3145,19 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor, U-VG Seminarier, U-G Projekt, U-VG Slutbetyget på kursen baseras på en helhetsbedö…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GIK2XK</t>
+          <t>GIK2XJ</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3178,19 +3178,19 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Duggor, U-VG Seminarier, U-G Projekt, U-VG Slutbetyget på kursen baseras på en helhetsbedö…</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XJ</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GIK2XZ</t>
+          <t>GIK2XK</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2022-09-27</t>
+          <t>2022-09-06</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
@@ -3216,14 +3216,14 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XK</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>IK1032</t>
+          <t>GIK2XZ</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2007-06-13</t>
+          <t>2022-09-27</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -3244,19 +3244,19 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XZ</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>IK1032</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3266,14 +3266,10 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2013-02-21</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>2014-09-01</t>
-        </is>
-      </c>
+          <t>2007-06-13</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>
           <t>Saknar punktlista</t>
@@ -3281,19 +3277,19 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter, laborati…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>IK1066</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3303,10 +3299,14 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2013-03-14</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
+          <t>2013-02-21</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>2014-09-01</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr">
         <is>
           <t>Saknar punktlista</t>
@@ -3314,29 +3314,29 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För seminarer används betygsskalan U-G samt för dugga och projektarbete betygsskalan U-VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetygets nivå fastställs genom en sammanvägning av inlämningsuppgifter, laborati…</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>GMA28W</t>
+          <t>IK1066</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2019-03-21</t>
+          <t>2013-03-14</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
@@ -3347,19 +3347,19 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För seminarer används betygsskalan U-G samt för dugga och projektarbete betygsskalan U-VG.…</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA28W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>GMA2EY</t>
+          <t>GMA28W</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>2020-03-04</t>
+          <t>2019-03-21</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -3380,19 +3380,19 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA28W</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>MA0011</t>
+          <t>GMA2EY</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2013-12-12</t>
+          <t>2020-03-04</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
@@ -3413,19 +3413,19 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen kräva att alla examinerande moment är godkän…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>MA0013</t>
+          <t>MA0011</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2014-01-30</t>
+          <t>2013-12-12</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
@@ -3446,19 +3446,19 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen krävs att alla examinerande moment är godkän…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen kräva att alla examinerande moment är godkän…</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0011</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>MA1040</t>
+          <t>MA0013</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2016-03-24</t>
+          <t>2014-01-30</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
@@ -3479,19 +3479,19 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg på kursen avgörs efter en sammanvägd bedömning av de enskilda tentamensres…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För att erhålla godkänt betyg på kursen krävs att alla examinerande moment är godkän…</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA0013</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>MA1042</t>
+          <t>MA1040</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3501,7 +3501,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2017-02-16</t>
+          <t>2016-03-24</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
@@ -3512,29 +3512,29 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg på kursen avgörs efter en sammanvägd bedömning av de enskilda tentamensres…</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1040</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>MA1042</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>2013-12-17</t>
+          <t>2017-02-16</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
@@ -3545,29 +3545,29 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla väl godkänt på kursen krävs väl godkänt som bedömning på 3 av 4 skriftliga…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>FMI2222</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MIKRODAT</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>2019-10-03</t>
+          <t>2013-12-17</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
@@ -3578,19 +3578,19 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla väl godkänt på kursen krävs väl godkänt som bedömning på 3 av 4 skriftliga…</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>FMI2223</t>
+          <t>FMI2222</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2017-10-04</t>
+          <t>2019-10-03</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
@@ -3616,14 +3616,14 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2223</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>FMI2224</t>
+          <t>FMI2223</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>2019-10-29</t>
+          <t>2017-10-04</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
@@ -3649,14 +3649,14 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2223</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>FMI2229</t>
+          <t>FMI2224</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2020-06-17</t>
+          <t>2019-10-29</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
@@ -3682,14 +3682,14 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2229</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>MIKR002</t>
+          <t>FMI2229</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2012-12-04</t>
+          <t>2020-06-17</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
@@ -3710,29 +3710,29 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Betygsrapportering: Moment 1: enskilt projekt 2 hp Moment 2: laborationsrapporter 1 hp Mome…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MIKR002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2229</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>MIKR002</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2018-04-05</t>
+          <t>2012-12-04</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
@@ -3743,19 +3743,19 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,G Workshop och inlämningsuppgifter, U,G. Seminarier U, 3,4,5 Skriftl…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G. Betygsrapportering: Moment 1: enskilt projekt 2 hp Moment 2: laborationsrapporter 1 hp Mome…</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MIKR002</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>GMT25Z</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3765,7 +3765,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2019-01-31</t>
+          <t>2018-04-05</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
@@ -3776,19 +3776,19 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,G Workshop och inlämningsuppgifter, U,G. Seminarier U, 3,4,5 Skriftl…</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>GMT25Z</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3798,7 +3798,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2021-05-20</t>
+          <t>2019-01-31</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
@@ -3809,19 +3809,19 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>MT1033</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3831,14 +3831,10 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2008-04-29</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>2010-08-26</t>
-        </is>
-      </c>
+          <t>2021-05-20</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr">
         <is>
           <t>Saknar punktlista</t>
@@ -3851,14 +3847,14 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>MT1033</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3868,10 +3864,14 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2014-04-03</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr"/>
+          <t>2008-04-29</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>2010-08-26</t>
+        </is>
+      </c>
       <c r="E104" t="inlineStr">
         <is>
           <t>Saknar punktlista</t>
@@ -3879,19 +3879,19 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2016-05-19</t>
+          <t>2014-04-03</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
@@ -3912,19 +3912,19 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Industriprojekt och workshop, U,G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>MT1074</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3934,7 +3934,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>2018-02-15</t>
+          <t>2016-05-19</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
@@ -3945,19 +3945,19 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer samt laborationsrapporter U-G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Industriprojekt och workshop, U,G.…</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>MT1074</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2007-05-22</t>
+          <t>2018-02-15</t>
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
@@ -3978,29 +3978,29 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationer samt laborationsrapporter U-G.…</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>2018-05-24</t>
+          <t>2007-05-22</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
@@ -4011,19 +4011,19 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2019-01-31</t>
+          <t>2018-05-24</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
@@ -4044,19 +4044,19 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntliga presentationer och skriftliga grupprapporter för projektet, U-G. Det samlade bety…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -4066,7 +4066,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>2019-06-05</t>
+          <t>2019-01-31</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
@@ -4077,19 +4077,19 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntliga presentationer och skriftliga grupprapporter för projektet, U-G. Det samlade bety…</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>AEG26X</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2021-05-20</t>
+          <t>2019-06-05</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
@@ -4110,19 +4110,19 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift 1: 2 hp, U-G Inlämningsuppgift 2: 3 hp, U, 3, 4, 5 Inlämningsuppgi…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>BEG222</t>
+          <t>AEG26X</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -4132,7 +4132,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2019-10-17</t>
+          <t>2021-05-20</t>
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
@@ -4143,19 +4143,19 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift 1: 2 hp, U-G Inlämningsuppgift 2: 3 hp, U, 3, 4, 5 Inlämningsuppgi…</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG26X</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>EG1012</t>
+          <t>BEG222</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2017-10-12</t>
+          <t>2019-10-17</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
@@ -4176,19 +4176,19 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts av examinator efter en sammanvägning av momenten.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>EG2004</t>
+          <t>EG1012</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -4198,7 +4198,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>2015-10-08</t>
+          <t>2017-10-12</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
@@ -4209,19 +4209,19 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Arbetet måste senast vara klart inom 18 månader från kursstart annars ges examensarb…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts av examinator efter en sammanvägning av momenten.…</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG2004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>EG2004</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>2015-08-27</t>
+          <t>2015-10-08</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
@@ -4242,19 +4242,19 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationsrapporter (U, G) Betyget för hela kursen sätts efter en samlad bedömning …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Arbetet måste senast vara klart inom 18 månader från kursstart annars ges examensarb…</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG2004</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>EG3009</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -4264,7 +4264,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>2015-09-17</t>
+          <t>2015-08-27</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
@@ -4275,19 +4275,19 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig hemuppgift 1, U-G. Slutbetyget sätts efter en samlad bedömning av examinat…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laborationsrapporter (U, G) Betyget för hela kursen sätts efter en samlad bedömning …</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>EG3012</t>
+          <t>EG3009</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -4308,19 +4308,19 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget för kursen är baserad på betyget för tentan…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Skriftlig hemuppgift 1, U-G. Slutbetyget sätts efter en samlad bedömning av examinat…</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3009</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>EG3012</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -4330,7 +4330,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2015-08-27</t>
+          <t>2015-09-17</t>
         </is>
       </c>
       <c r="D118" t="inlineStr"/>
@@ -4341,19 +4341,19 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter bedömning av reflektionsprotokoll. Väl genomförda skriftliga r…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyget för kursen är baserad på betyget för tentan…</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>EG3014</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -4374,19 +4374,19 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Reflektionsprotokoll, skriftlig rapport och projektuppgift (U-G). Den skiftliga tent…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter bedömning av reflektionsprotokoll. Väl genomförda skriftliga r…</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>EG3017</t>
+          <t>EG3015</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -4396,7 +4396,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2016-09-22</t>
+          <t>2015-08-27</t>
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
@@ -4407,19 +4407,19 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Reflektionsprotokoll, skriftlig rapport och projektuppgift (U-G). Den skiftliga tent…</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>EG3018</t>
+          <t>EG3017</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -4445,14 +4445,14 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>EG3019</t>
+          <t>EG3018</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>2017-04-27</t>
+          <t>2016-09-22</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -4473,19 +4473,19 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laboration och Inlämningsuppgifter U,G…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3019</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>EG3020</t>
+          <t>EG3019</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2017-12-14</t>
+          <t>2017-04-27</t>
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
@@ -4506,19 +4506,19 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Laboration och Inlämningsuppgifter U,G…</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3019</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>EG3022</t>
+          <t>EG3020</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>2018-01-25</t>
+          <t>2017-12-14</t>
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
@@ -4539,19 +4539,19 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5.…</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3020</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>EG4001</t>
+          <t>EG3022</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>2014-11-27</t>
+          <t>2018-01-25</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
@@ -4577,14 +4577,14 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>EG4001</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2014-11-27</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
@@ -4605,19 +4605,19 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F.…</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>GEG2JP</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>2020-09-24</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="D127" t="inlineStr"/>
@@ -4638,19 +4638,19 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift, rapport och muntlig presentation ger U eller G. Det samlade betyg…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>GEG2UE</t>
+          <t>GEG2JP</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>2022-01-27</t>
+          <t>2020-09-24</t>
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
@@ -4671,19 +4671,19 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Rapporter (U/G) Betygssättning av kursen sker genom den skriftliga salstentamen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Inlämningsuppgift, rapport och muntlig presentation ger U eller G. Det samlade betyg…</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>GEG2UL</t>
+          <t>GEG2UE</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2022-01-27</t>
         </is>
       </c>
       <c r="D129" t="inlineStr"/>
@@ -4704,29 +4704,29 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntlig redovisning U-G. Projekt U-VG. Kursens slutbetyg baseras på en samlad bedömning av…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Rapporter (U/G) Betygssättning av kursen sker genom den skriftliga salstentamen.…</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UE</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>GSQ23J</t>
+          <t>GEG2UL</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>2018-05-24</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="D130" t="inlineStr"/>
@@ -4737,19 +4737,19 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Muntlig redovisning U-G. Projekt U-VG. Kursens slutbetyg baseras på en samlad bedömning av…</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GSQ23J</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -4759,7 +4759,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>2018-06-14</t>
+          <t>2018-05-24</t>
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
@@ -4770,19 +4770,19 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,VG Slutbetyget på kursen sätts efter en samlad bedömning av examinat…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>GSQ25F</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -4792,7 +4792,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>2018-10-29</t>
+          <t>2018-06-14</t>
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
@@ -4803,19 +4803,19 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete och övningsuppgifter U,VG. Slutbetyget utgör en sammanvägning av betyg…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete U,VG Slutbetyget på kursen sätts efter en samlad bedömning av examinat…</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>GSQ25J</t>
+          <t>GSQ25F</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -4836,19 +4836,19 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Projektarbete och övningsuppgifter U,VG. Slutbetyget utgör en sammanvägning av betyg…</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25F</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>GSQ25K</t>
+          <t>GSQ25J</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -4858,7 +4858,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2018-11-08</t>
+          <t>2018-10-29</t>
         </is>
       </c>
       <c r="D134" t="inlineStr"/>
@@ -4869,19 +4869,19 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För projektarbetet är betygsskalan U,G,VG. Slutbetyget på kursen sätts efter en saml…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>GSQ25N</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -4902,19 +4902,19 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För projektarbetet är betygsskalan U,G,VG. Slutbetyget på kursen sätts efter en saml…</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>GSQ25N</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2020-02-06</t>
+          <t>2018-11-08</t>
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
@@ -4935,19 +4935,19 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25N</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>GSQ2H7</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>2020-06-29</t>
+          <t>2020-02-06</t>
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
@@ -4968,19 +4968,19 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>GSQ2J4</t>
+          <t>GSQ2H7</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -4990,7 +4990,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>2020-09-03</t>
+          <t>2020-06-29</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
@@ -5001,19 +5001,19 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som sammanvägd betygsskala används U, 3,4, 5 med följande fördelning på delmomenten:…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L8</t>
+          <t>GSQ2J4</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2020-12-17</t>
+          <t>2020-09-03</t>
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
@@ -5034,19 +5034,19 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Tentamen och seminarier med skriftliga inlämningar, U, 3, 4, 5. Projektuppgiften, U,…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som sammanvägd betygsskala används U, 3,4, 5 med följande fördelning på delmomenten:…</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2J4</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>GSQ2L8</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5067,19 +5067,19 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Tentamen och seminarier med skriftliga inlämningar, U, 3, 4, 5. Projektuppgiften, U,…</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L8</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>GSQ2LA</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -5100,19 +5100,19 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Tentamen och övningar, U-G. Seminarier och projektuppgift, U-VG. Slutbetyget på kursen sät…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2LA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>GSQ2MC</t>
+          <t>GSQ2LA</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>2021-02-18</t>
+          <t>2020-12-17</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -5133,19 +5133,19 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter en samlad bedömning av examinator.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Tentamen och övningar, U-G. Seminarier och projektuppgift, U-VG. Slutbetyget på kursen sät…</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2LA</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>GSQ2PH</t>
+          <t>GSQ2MC</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -5155,7 +5155,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
+          <t>2021-02-18</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
@@ -5166,19 +5166,19 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som betygsskala för kursen och för tentamen används U, 3, 4, 5. För litteratursemina…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Slutbetyg sätts efter en samlad bedömning av examinator.…</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>GSQ2R5</t>
+          <t>GSQ2PH</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -5188,7 +5188,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2021-08-24</t>
+          <t>2021-04-15</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
@@ -5199,19 +5199,19 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U-VG) Övningar (U-G) Seminarier (U-G)…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. Som betygsskala för kursen och för tentamen används U, 3, 4, 5. För litteratursemina…</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2R5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>GSQ2VY</t>
+          <t>GSQ2R5</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>2022-03-24</t>
+          <t>2021-08-24</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
@@ -5232,19 +5232,19 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektet styr slutbetyget på kursen.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete (U-VG) Övningar (U-G) Seminarier (U-G)…</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2R5</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>GSQ2WM</t>
+          <t>GSQ2VY</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -5254,7 +5254,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2022-06-08</t>
+          <t>2022-03-24</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -5265,19 +5265,19 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på Modul 1 och Modul 2. Modul 1: Kartografi och …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektet styr slutbetyget på kursen.…</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>GSQ2Y2</t>
+          <t>GSQ2WM</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>2022-09-27</t>
+          <t>2022-06-08</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -5298,19 +5298,19 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på både Modul 1 och Modul 2. Modul 1: Kvalitativ…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på Modul 1 och Modul 2. Modul 1: Kartografi och …</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2Y2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>SQ1003</t>
+          <t>GSQ2Y2</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>2017-10-12</t>
+          <t>2022-09-27</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -5331,29 +5331,29 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För betyget VG på kursen krävs betyget VG på både Modul 1 och Modul 2. Modul 1: Kvalitativ…</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2Y2</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>GST2CL</t>
+          <t>SQ1003</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2020-01-30</t>
+          <t>2017-10-12</t>
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
@@ -5364,19 +5364,19 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U, 3, 4, 5. För högre betyg än 3 på kursen krävs högre betyg än 3 på både de kvalitativa och kva…</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>ST1013</t>
+          <t>GST2CL</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -5386,14 +5386,10 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>2010-12-14</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>2013-02-13</t>
-        </is>
-      </c>
+          <t>2020-01-30</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
       <c r="E150" t="inlineStr">
         <is>
           <t>Saknar punktlista</t>
@@ -5406,27 +5402,31 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>AMI22T</t>
+          <t>ST1013</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr"/>
+          <t>2010-12-14</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>2013-02-13</t>
+        </is>
+      </c>
       <c r="E151" t="inlineStr">
         <is>
           <t>Saknar punktlista</t>
@@ -5439,14 +5439,14 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>AMI22Z</t>
+          <t>AMI22T</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>2019-04-18</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="D152" t="inlineStr"/>
@@ -5467,19 +5467,19 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22T</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>AMI23A</t>
+          <t>AMI22Z</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>2019-08-29</t>
+          <t>2019-04-18</t>
         </is>
       </c>
       <c r="D153" t="inlineStr"/>
@@ -5500,19 +5500,19 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI22Z</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>AMI23C</t>
+          <t>AMI23A</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -5533,19 +5533,19 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23A</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>AMI23G</t>
+          <t>AMI23C</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -5555,7 +5555,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>2019-10-17</t>
+          <t>2019-08-29</t>
         </is>
       </c>
       <c r="D155" t="inlineStr"/>
@@ -5566,19 +5566,19 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete U - VG Laborationer, seminarier och skriftlig reflektioner U-G. Slutbetyget …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23C</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>AMI23J</t>
+          <t>AMI23G</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -5588,7 +5588,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>2019-11-07</t>
+          <t>2019-10-17</t>
         </is>
       </c>
       <c r="D156" t="inlineStr"/>
@@ -5599,19 +5599,19 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Projektarbete U - VG Laborationer, seminarier och skriftlig reflektioner U-G. Slutbetyget …</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23G</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>AMI23K</t>
+          <t>AMI23J</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -5621,7 +5621,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2019-10-17</t>
+          <t>2019-11-07</t>
         </is>
       </c>
       <c r="D157" t="inlineStr"/>
@@ -5632,19 +5632,19 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget på kursen sätts efter en samlad bedömning av examina…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23J</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>AMI23L</t>
+          <t>AMI23K</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -5665,19 +5665,19 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Laborationsrapporter U-G. Slutbetyget på kursen sätts efter en samlad bedömning av examina…</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23K</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>AMI27V</t>
+          <t>AMI23L</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2019-10-17</t>
         </is>
       </c>
       <c r="D159" t="inlineStr"/>
@@ -5698,19 +5698,19 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG.…</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI27V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI23L</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>GMI23G</t>
+          <t>AMI27V</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>2018-06-14</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="D160" t="inlineStr"/>
@@ -5731,19 +5731,19 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Slutbetyget på kursen baseras på en helhetsbedömning av examinatorn.…</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMI27V</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>GMI24H</t>
+          <t>GMI23G</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -5753,7 +5753,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2018-09-13</t>
+          <t>2018-06-14</t>
         </is>
       </c>
       <c r="D161" t="inlineStr"/>
@@ -5764,19 +5764,19 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Labborationsuppgifter U-G Salstentamen U-VG Kursens slutbetyg bestäms av betyget för salst…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>GMI26H</t>
+          <t>GMI24H</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2018-09-13</t>
         </is>
       </c>
       <c r="D162" t="inlineStr"/>
@@ -5797,19 +5797,19 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betygets nivå fastställs genom tentamen, vilket också blir slutbetyget under förutsättning…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Labborationsuppgifter U-G Salstentamen U-VG Kursens slutbetyg bestäms av betyget för salst…</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>GMI2C8</t>
+          <t>GMI26H</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -5819,7 +5819,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>2019-10-17</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="D163" t="inlineStr"/>
@@ -5830,19 +5830,19 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betygets nivå fastställs genom tentamen, vilket också blir slutbetyget under förutsättning…</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>GMI2J3</t>
+          <t>GMI2C8</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -5852,7 +5852,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>2020-09-03</t>
+          <t>2019-10-17</t>
         </is>
       </c>
       <c r="D164" t="inlineStr"/>
@@ -5863,19 +5863,19 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Inlämningsuppgifter och gruppresentation, U-G. Skriftlig tentamen, U-VG.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. För att erhålla VG som slutbetyg på kursen krävs att bedömningskriterier för VG uppfylls s…</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>GMI2MD</t>
+          <t>GMI2J3</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -5885,7 +5885,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2021-02-18</t>
+          <t>2020-09-03</t>
         </is>
       </c>
       <c r="D165" t="inlineStr"/>
@@ -5896,19 +5896,19 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Individuell muntlig och skriftlig redovisning av inlämningsuppgifter och gruppresentation …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Inlämningsuppgifter och gruppresentation, U-G. Skriftlig tentamen, U-VG.…</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>GMI2NW</t>
+          <t>GMI2MD</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -5918,7 +5918,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>2021-03-11</t>
+          <t>2021-02-18</t>
         </is>
       </c>
       <c r="D166" t="inlineStr"/>
@@ -5929,19 +5929,19 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Individuell muntlig och skriftlig redovisning av inlämningsuppgifter och gruppresentation …</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2NW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2MD</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>MI4001</t>
+          <t>GMI2NW</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -5951,14 +5951,10 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>2011-02-15</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>2012-11-07</t>
-        </is>
-      </c>
+          <t>2021-03-11</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
       <c r="E167" t="inlineStr">
         <is>
           <t>Saknar punktlista</t>
@@ -5966,50 +5962,87 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget är individuellt och sätts på grundval av det material som föreligger vid slutsemin…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–G.…</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2NW</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
+          <t>MI4001</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>2011-02-15</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>2012-11-07</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget är individuellt och sätts på grundval av det material som föreligger vid slutsemin…</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4001</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
           <t>MI4002</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr">
+      <c r="B169" t="inlineStr">
         <is>
           <t>XYZ</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr">
+      <c r="C169" t="inlineStr">
         <is>
           <t>2011-12-08</t>
         </is>
       </c>
-      <c r="D168" t="inlineStr"/>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>Saknar punktlista</t>
-        </is>
-      </c>
-      <c r="F168" t="inlineStr">
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Saknar punktlista</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
         <is>
           <t>Betyg skrivet utan punktlista: Som betygsskala används U–VG. Betyget är individuellt och sätts på grundval av det material som föreligger vid slutsemin…</t>
         </is>
       </c>
-      <c r="G168" s="2" t="inlineStr">
+      <c r="G169" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MI4002</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G168"/>
+  <autoFilter ref="A1:G169"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -6345,6 +6378,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G167" r:id="rId332"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A168" r:id="rId333"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G168" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A169" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G169" r:id="rId336"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>